<commit_message>
update výpisu a zadání
</commit_message>
<xml_diff>
--- a/Zadání.xlsx
+++ b/Zadání.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20375"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\2.RP_2023\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Xampp\htdocs\2.RP_2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DFF3221-8C0C-4CDE-95CF-939C27253278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F873BEA-F421-425D-A631-1A49BE59DF16}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,17 +22,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -413,15 +402,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -527,7 +516,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="cs-CZ"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -628,13 +617,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>23</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -691,7 +680,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="cs-CZ"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -721,7 +710,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="en-US"/>
+      <a:endParaRPr lang="cs-CZ"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -1609,11 +1598,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
@@ -1685,7 +1674,7 @@
       </c>
       <c r="J4">
         <f>COUNTIF(E3:E33,"ne")</f>
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -1741,7 +1730,7 @@
       </c>
       <c r="J6">
         <f>COUNTIF(E3:E33,"ano")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -1769,7 +1758,7 @@
       </c>
       <c r="J7">
         <f>SUM(F3:F33)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -2030,7 +2019,7 @@
       <c r="D21" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" s="13" t="s">
         <v>50</v>
       </c>
       <c r="F21">
@@ -2051,7 +2040,7 @@
       <c r="D22" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E22" s="16" t="s">
+      <c r="E22" s="14" t="s">
         <v>50</v>
       </c>
       <c r="F22">
@@ -2072,7 +2061,7 @@
       <c r="D23" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E23" s="16" t="s">
+      <c r="E23" s="14" t="s">
         <v>50</v>
       </c>
       <c r="F23">
@@ -2093,7 +2082,7 @@
       <c r="D24" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="15" t="s">
         <v>50</v>
       </c>
       <c r="F24">
@@ -2122,12 +2111,12 @@
       <c r="D26" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E26" s="15" t="s">
-        <v>41</v>
+      <c r="E26" s="13" t="s">
+        <v>50</v>
       </c>
       <c r="F26">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2141,12 +2130,12 @@
       <c r="D27" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="E27" s="16" t="s">
-        <v>41</v>
+      <c r="E27" s="14" t="s">
+        <v>50</v>
       </c>
       <c r="F27">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2162,7 +2151,7 @@
       <c r="D28" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E28" s="16" t="s">
+      <c r="E28" s="14" t="s">
         <v>41</v>
       </c>
       <c r="F28">
@@ -2262,14 +2251,14 @@
     </row>
     <row r="34" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
-      <c r="B34" s="13"/>
+      <c r="B34" s="16"/>
       <c r="C34" s="5" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
-      <c r="B35" s="13"/>
+      <c r="B35" s="16"/>
       <c r="C35" s="5" t="s">
         <v>32</v>
       </c>

</xml_diff>

<commit_message>
přidání placeholderů do vyhledávače
</commit_message>
<xml_diff>
--- a/Zadání.xlsx
+++ b/Zadání.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10514"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20396"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/XAMPP/xamppfiles/htdocs/cinedb/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\cinedb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7E25618-42C0-6A43-8378-A30FC7F31ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A99657DA-EE0D-4223-8F66-5CCAC8F071BE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="495" windowWidth="28800" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -22,17 +22,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -252,7 +241,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -262,6 +251,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -394,7 +389,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -425,6 +420,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -631,13 +627,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>7</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>15</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1599,26 +1595,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="3.5" customWidth="1"/>
-    <col min="3" max="3" width="77.83203125" customWidth="1"/>
-    <col min="4" max="4" width="17.5" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.33203125" customWidth="1"/>
-    <col min="7" max="7" width="51.1640625" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.42578125" customWidth="1"/>
+    <col min="3" max="3" width="77.85546875" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.28515625" customWidth="1"/>
+    <col min="7" max="7" width="51.140625" customWidth="1"/>
+    <col min="9" max="9" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="17" t="s">
         <v>17</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>35</v>
       </c>
@@ -1635,7 +1631,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -1660,10 +1656,10 @@
       </c>
       <c r="J3">
         <f>COUNTIF(E3:E33,"ano")+COUNTIF(E3:E33,"ne")</f>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1688,10 +1684,10 @@
       </c>
       <c r="J4">
         <f>COUNTIF(E3:E33,"ne")</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -1716,10 +1712,10 @@
       </c>
       <c r="J5">
         <f>COUNTIF(E3:E33,"wip")</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
@@ -1744,10 +1740,10 @@
       </c>
       <c r="J6">
         <f>COUNTIF(E3:E33,"ano")</f>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>2</v>
       </c>
@@ -1772,10 +1768,10 @@
       </c>
       <c r="J7">
         <f>SUM(F3:F33)</f>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>2</v>
       </c>
@@ -1796,7 +1792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>2</v>
       </c>
@@ -1817,7 +1813,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>2</v>
       </c>
@@ -1838,7 +1834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2">
         <v>1</v>
@@ -1857,7 +1853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="4">
         <f>SUM(B3:B11)</f>
@@ -1865,7 +1861,7 @@
       </c>
       <c r="C12" s="3"/>
     </row>
-    <row r="13" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>3</v>
       </c>
@@ -1886,7 +1882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>3</v>
       </c>
@@ -1907,7 +1903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>3</v>
       </c>
@@ -1928,7 +1924,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>3</v>
       </c>
@@ -1949,7 +1945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>3</v>
       </c>
@@ -1970,7 +1966,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>3</v>
       </c>
@@ -1991,7 +1987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>3</v>
       </c>
@@ -2012,7 +2008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="4">
         <f>SUM(B13:B19)</f>
@@ -2020,7 +2016,7 @@
       </c>
       <c r="C20" s="3"/>
     </row>
-    <row r="21" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>4</v>
       </c>
@@ -2041,7 +2037,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>4</v>
       </c>
@@ -2062,7 +2058,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>4</v>
       </c>
@@ -2083,7 +2079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>4</v>
       </c>
@@ -2104,7 +2100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="4">
         <f>SUM(B21:B24)</f>
@@ -2112,7 +2108,7 @@
       </c>
       <c r="C25" s="3"/>
     </row>
-    <row r="26" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>10</v>
       </c>
@@ -2133,7 +2129,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="2">
         <v>1</v>
@@ -2152,7 +2148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>10</v>
       </c>
@@ -2173,7 +2169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>6</v>
       </c>
@@ -2186,15 +2182,15 @@
       <c r="D29" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E29" s="8" t="s">
-        <v>41</v>
+      <c r="E29" s="18" t="s">
+        <v>51</v>
       </c>
       <c r="F29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>6</v>
       </c>
@@ -2208,14 +2204,14 @@
         <v>39</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="F30">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>10</v>
       </c>
@@ -2236,7 +2232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="4">
         <f>SUM(B26:B31)</f>
@@ -2244,7 +2240,7 @@
       </c>
       <c r="C32" s="3"/>
     </row>
-    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="4">
         <v>2</v>
@@ -2263,21 +2259,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="16"/>
       <c r="C34" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="16"/>
       <c r="C35" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="6"/>

</xml_diff>